<commit_message>
FIX: test for #4562 silently not passing.
</commit_message>
<xml_diff>
--- a/docs/lexer/lexer-FSM.xlsx
+++ b/docs/lexer/lexer-FSM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Red\docs\lexer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8484D164-720B-4F9B-ADF0-1C22A15EC6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AE920D-BFFE-4EEB-9F1E-EF3F3F224E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5140" yWindow="1080" windowWidth="18080" windowHeight="18840" tabRatio="564" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="430" yWindow="20" windowWidth="34400" windowHeight="20750" tabRatio="564" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="transitions" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2760" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2801" uniqueCount="160">
   <si>
     <t>S_START</t>
   </si>
@@ -498,6 +498,9 @@
   </si>
   <si>
     <t>S_FL_DEC1</t>
+  </si>
+  <si>
+    <t>S_SIGN_W</t>
   </si>
 </sst>
 </file>
@@ -967,7 +970,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AO65"/>
+  <dimension ref="A1:AO66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.36328125" style="7" bestFit="1" customWidth="1"/>
@@ -7104,7 +7107,7 @@
     </row>
     <row r="50" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
-        <v>106</v>
+        <v>159</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>72</v>
@@ -7113,10 +7116,10 @@
         <v>72</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>72</v>
@@ -7142,11 +7145,11 @@
       <c r="M50" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="N50" s="2" t="s">
-        <v>30</v>
+      <c r="N50" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="O50" s="2" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="P50" s="2" t="s">
         <v>30</v>
@@ -7187,14 +7190,14 @@
       <c r="AB50" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AC50" s="3" t="s">
-        <v>60</v>
+      <c r="AC50" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="AD50" s="1" t="s">
         <v>72</v>
       </c>
       <c r="AE50" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="AF50" s="2" t="s">
         <v>30</v>
@@ -7203,13 +7206,13 @@
         <v>60</v>
       </c>
       <c r="AH50" s="2" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="AI50" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="AJ50" s="2" t="s">
-        <v>30</v>
+        <v>30</v>
+      </c>
+      <c r="AJ50" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AK50" s="1" t="s">
         <v>72</v>
@@ -7229,13 +7232,13 @@
     </row>
     <row r="51" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>107</v>
@@ -7244,85 +7247,85 @@
         <v>107</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="M51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="N51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="O51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
+      </c>
+      <c r="M51" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="P51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="R51" s="3" t="s">
-        <v>60</v>
+        <v>30</v>
+      </c>
+      <c r="Q51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="R51" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="T51" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="U51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="V51" s="3" t="s">
-        <v>60</v>
+        <v>30</v>
+      </c>
+      <c r="U51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V51" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="W51" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="X51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y51" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="Z51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB51" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
+      </c>
+      <c r="X51" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB51" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AC51" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD51" s="3" t="s">
-        <v>60</v>
+      <c r="AD51" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="AE51" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AF51" s="3" t="s">
-        <v>60</v>
+      <c r="AF51" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="AG51" s="3" t="s">
         <v>60</v>
@@ -7333,61 +7336,61 @@
       <c r="AI51" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="AJ51" s="3" t="s">
-        <v>60</v>
+      <c r="AJ51" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="AK51" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AL51" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM51" s="3" t="s">
-        <v>60</v>
+        <v>72</v>
+      </c>
+      <c r="AL51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AM51" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="AN51" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AO51" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="K52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="L52" s="3" t="s">
-        <v>60</v>
+        <v>107</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="M52" s="3" t="s">
         <v>60</v>
@@ -7395,47 +7398,47 @@
       <c r="N52" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="O52" s="3" t="s">
-        <v>60</v>
+      <c r="O52" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="P52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="R52" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
+      </c>
+      <c r="Q52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R52" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="U52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="V52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W52" s="2" t="s">
-        <v>148</v>
+        <v>107</v>
+      </c>
+      <c r="U52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="V52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="W52" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="X52" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="Y52" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Z52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA52" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="AB52" s="4" t="s">
-        <v>144</v>
+      <c r="Y52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB52" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="AC52" s="3" t="s">
         <v>60</v>
@@ -7443,85 +7446,85 @@
       <c r="AD52" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AE52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AF52" s="2" t="s">
-        <v>30</v>
+      <c r="AE52" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF52" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AG52" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AH52" s="2" t="s">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="AI52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AJ52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AK52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL52" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AM52" s="2" t="s">
-        <v>30</v>
+        <v>107</v>
+      </c>
+      <c r="AJ52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK52" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM52" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AN52" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO52" s="3" t="s">
-        <v>60</v>
+      <c r="AO52" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N53" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O53" s="2" t="s">
-        <v>92</v>
+        <v>119</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="N53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O53" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="P53" s="2" t="s">
         <v>30</v>
@@ -7544,50 +7547,50 @@
       <c r="V53" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="W53" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="X53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y53" s="1" t="s">
-        <v>72</v>
+      <c r="W53" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="X53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y53" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="Z53" s="2" t="s">
         <v>30</v>
       </c>
       <c r="AA53" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB53" s="3" t="s">
-        <v>60</v>
+        <v>150</v>
+      </c>
+      <c r="AB53" s="4" t="s">
+        <v>144</v>
       </c>
       <c r="AC53" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AE53" s="2" t="s">
-        <v>21</v>
+      <c r="AD53" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE53" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AF53" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AG53" s="2" t="s">
-        <v>22</v>
+      <c r="AG53" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AH53" s="2" t="s">
-        <v>30</v>
+        <v>159</v>
       </c>
       <c r="AI53" s="2" t="s">
-        <v>30</v>
+        <v>159</v>
       </c>
       <c r="AJ53" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AK53" s="1" t="s">
-        <v>72</v>
+      <c r="AK53" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AL53" s="2" t="s">
         <v>30</v>
@@ -7598,127 +7601,127 @@
       <c r="AN53" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO53" s="1" t="s">
-        <v>72</v>
+      <c r="AO53" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="54" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A54" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O54" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="N54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="O54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="P54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="R54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="S54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="T54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="U54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="V54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="W54" s="4" t="s">
-        <v>31</v>
+      <c r="P54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="R54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="T54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="U54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W54" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="X54" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="Y54" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AA54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC54" s="4" t="s">
-        <v>31</v>
+      <c r="Y54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB54" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC54" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AD54" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AE54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AF54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AI54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AJ54" s="4" t="s">
-        <v>31</v>
+      <c r="AE54" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG54" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AH54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AI54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AJ54" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="AK54" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AL54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AM54" s="4" t="s">
-        <v>31</v>
+      <c r="AL54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AM54" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="AN54" s="3" t="s">
         <v>60</v>
@@ -7729,7 +7732,7 @@
     </row>
     <row r="55" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
-        <v>144</v>
+        <v>92</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>72</v>
@@ -7737,11 +7740,11 @@
       <c r="C55" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>60</v>
+      <c r="D55" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>72</v>
@@ -7761,41 +7764,41 @@
       <c r="K55" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="L55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="M55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="N55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="O55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="P55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="R55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="S55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="T55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="U55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="V55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="W55" s="3" t="s">
-        <v>60</v>
+      <c r="L55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="S55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="T55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="U55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="V55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="W55" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="X55" s="1" t="s">
         <v>72</v>
@@ -7803,47 +7806,47 @@
       <c r="Y55" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="Z55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA55" s="3" t="s">
-        <v>60</v>
+      <c r="Z55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA55" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="AB55" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="AC55" s="3" t="s">
-        <v>60</v>
+        <v>31</v>
+      </c>
+      <c r="AC55" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="AD55" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AE55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AF55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ55" s="3" t="s">
-        <v>60</v>
+      <c r="AE55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AI55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AJ55" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="AK55" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AL55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM55" s="3" t="s">
-        <v>60</v>
+      <c r="AL55" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AM55" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="AN55" s="3" t="s">
         <v>60</v>
@@ -7854,290 +7857,290 @@
     </row>
     <row r="56" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="s">
-        <v>31</v>
+        <v>144</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>31</v>
+        <v>72</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="L56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="R56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="U56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="V56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="W56" s="2" t="s">
-        <v>31</v>
+        <v>72</v>
+      </c>
+      <c r="L56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="N56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="S56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="T56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="U56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="V56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="W56" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="X56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="Y56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
+      </c>
+      <c r="Y56" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="Z56" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AA56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC56" s="2" t="s">
-        <v>31</v>
+      <c r="AA56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB56" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC56" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AD56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="AE56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AF56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AI56" s="2" t="s">
-        <v>31</v>
+        <v>72</v>
+      </c>
+      <c r="AE56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI56" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AJ56" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AK56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AM56" s="2" t="s">
-        <v>31</v>
+        <v>72</v>
+      </c>
+      <c r="AL56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM56" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AN56" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AO56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
     </row>
     <row r="57" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="M57" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="N57" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="O57" s="3" t="s">
-        <v>60</v>
+        <v>90</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="P57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="Q57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="R57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="S57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="T57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="U57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="V57" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="W57" s="1" t="s">
-        <v>93</v>
+        <v>31</v>
+      </c>
+      <c r="W57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="X57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Y57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Z57" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AA57" s="3" t="s">
-        <v>60</v>
+      <c r="AA57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="AB57" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC57" s="3" t="s">
-        <v>60</v>
+        <v>31</v>
+      </c>
+      <c r="AC57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="AD57" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AE57" s="3" t="s">
-        <v>60</v>
+        <v>90</v>
+      </c>
+      <c r="AE57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="AF57" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG57" s="3" t="s">
-        <v>60</v>
+        <v>31</v>
+      </c>
+      <c r="AG57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="AH57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="AI57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="AJ57" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AK57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="AL57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="AM57" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="AN57" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AO57" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="58" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>60</v>
@@ -8145,38 +8148,38 @@
       <c r="N58" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="O58" s="2" t="s">
-        <v>145</v>
+      <c r="O58" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="P58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="Q58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="R58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="S58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="T58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="U58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="V58" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="W58" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="X58" s="3" t="s">
-        <v>60</v>
+        <v>21</v>
+      </c>
+      <c r="W58" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="X58" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="Y58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="Z58" s="3" t="s">
         <v>60</v>
@@ -8185,254 +8188,254 @@
         <v>60</v>
       </c>
       <c r="AB58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="AC58" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AD58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="AE58" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AF58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="AG58" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AH58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="AI58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="AJ58" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AK58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
       <c r="AL58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="AM58" s="2" t="s">
-        <v>145</v>
+        <v>21</v>
       </c>
       <c r="AN58" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AO58" s="1" t="s">
-        <v>146</v>
+        <v>93</v>
       </c>
     </row>
     <row r="59" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="M59" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="N59" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O59" s="1" t="s">
-        <v>72</v>
+      <c r="N59" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="P59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="Q59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="R59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="S59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="T59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="U59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="V59" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W59" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="X59" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y59" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z59" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA59" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB59" s="3" t="s">
-        <v>60</v>
+        <v>145</v>
+      </c>
+      <c r="W59" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="X59" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y59" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z59" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA59" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB59" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="AC59" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AD59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="AE59" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AF59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="AG59" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AH59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="AI59" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AJ59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
+      </c>
+      <c r="AJ59" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AK59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="AL59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="AM59" s="2" t="s">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="AN59" s="3" t="s">
         <v>60</v>
       </c>
       <c r="AO59" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
     </row>
     <row r="60" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>60</v>
+        <v>150</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>60</v>
+        <v>30</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="J60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="K60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>99</v>
+        <v>72</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L60" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M60" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="O60" s="2" t="s">
-        <v>120</v>
+        <v>30</v>
+      </c>
+      <c r="O60" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="P60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="Q60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="R60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="S60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="T60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="U60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="W60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="X60" s="3" t="s">
-        <v>60</v>
+        <v>30</v>
+      </c>
+      <c r="W60" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="X60" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="Y60" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="Z60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="AA60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="AB60" s="3" t="s">
         <v>60</v>
@@ -8440,52 +8443,52 @@
       <c r="AC60" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE60" s="2" t="s">
-        <v>145</v>
+      <c r="AD60" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE60" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AF60" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AG60" s="2" t="s">
-        <v>22</v>
+        <v>30</v>
+      </c>
+      <c r="AG60" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AH60" s="2" t="s">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="AI60" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="AJ60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AK60" s="3" t="s">
-        <v>60</v>
+        <v>30</v>
+      </c>
+      <c r="AJ60" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AK60" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="AL60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="AM60" s="2" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="AN60" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO60" s="3" t="s">
-        <v>60</v>
+      <c r="AO60" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="61" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A61" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>80</v>
+        <v>96</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>97</v>
@@ -8493,285 +8496,285 @@
       <c r="E61" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>80</v>
+      <c r="F61" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="L61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M61" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
+      </c>
+      <c r="J61" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K61" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="O61" s="1" t="s">
-        <v>80</v>
+        <v>120</v>
+      </c>
+      <c r="O61" s="2" t="s">
+        <v>120</v>
       </c>
       <c r="P61" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="R61" s="3" t="s">
-        <v>60</v>
+        <v>98</v>
+      </c>
+      <c r="Q61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="R61" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="S61" s="2" t="s">
-        <v>138</v>
+        <v>98</v>
       </c>
       <c r="T61" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="U61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="V61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="W61" s="1" t="s">
-        <v>80</v>
+        <v>98</v>
+      </c>
+      <c r="U61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="V61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="W61" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="X61" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="Y61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="Z61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB61" s="1" t="s">
-        <v>81</v>
+      <c r="Y61" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB61" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AC61" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD61" s="1" t="s">
-        <v>80</v>
+      <c r="AD61" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AE61" s="2" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="AF61" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AG61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI61" s="3" t="s">
-        <v>60</v>
+        <v>98</v>
+      </c>
+      <c r="AG61" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AH61" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI61" s="2" t="s">
+        <v>100</v>
       </c>
       <c r="AJ61" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AK61" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="AL61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM61" s="3" t="s">
-        <v>60</v>
+      <c r="AK61" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL61" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AM61" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="AN61" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO61" s="1" t="s">
-        <v>80</v>
+      <c r="AO61" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A62" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="K62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="L62" s="3" t="s">
-        <v>60</v>
+        <v>97</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="M62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="N62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="O62" s="3" t="s">
-        <v>60</v>
+      <c r="N62" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="O62" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="P62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="Q62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="R62" s="2" t="s">
-        <v>98</v>
+        <v>19</v>
+      </c>
+      <c r="Q62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R62" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="S62" s="2" t="s">
-        <v>98</v>
+        <v>138</v>
       </c>
       <c r="T62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="U62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="V62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="W62" s="3" t="s">
-        <v>60</v>
+        <v>138</v>
+      </c>
+      <c r="U62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="V62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="W62" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="X62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="Y62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="Z62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AB62" s="3" t="s">
-        <v>60</v>
+      <c r="Y62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="Z62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB62" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="AC62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE62" s="3" t="s">
-        <v>60</v>
+      <c r="AD62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE62" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="AF62" s="2" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="AG62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AH62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AI62" s="2" t="s">
-        <v>98</v>
+      <c r="AH62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI62" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AJ62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AK62" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL62" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM62" s="2" t="s">
-        <v>98</v>
+      <c r="AK62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AL62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM62" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AN62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO62" s="3" t="s">
-        <v>60</v>
+      <c r="AO62" s="1" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="63" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A63" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L63" s="1" t="s">
-        <v>72</v>
+        <v>120</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L63" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="M63" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="N63" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="O63" s="1" t="s">
-        <v>72</v>
+      <c r="N63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O63" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="P63" s="2" t="s">
         <v>98</v>
@@ -8794,11 +8797,11 @@
       <c r="V63" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="W63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="X63" s="1" t="s">
-        <v>72</v>
+      <c r="W63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="X63" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="Y63" s="2" t="s">
         <v>98</v>
@@ -8815,17 +8818,17 @@
       <c r="AC63" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD63" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AE63" s="2" t="s">
-        <v>21</v>
+      <c r="AD63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE63" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AF63" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AG63" s="2" t="s">
-        <v>22</v>
+      <c r="AG63" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AH63" s="2" t="s">
         <v>98</v>
@@ -8833,11 +8836,11 @@
       <c r="AI63" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AJ63" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AK63" s="1" t="s">
-        <v>72</v>
+      <c r="AJ63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK63" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AL63" s="2" t="s">
         <v>98</v>
@@ -8848,257 +8851,382 @@
       <c r="AN63" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO63" s="1" t="s">
-        <v>72</v>
+      <c r="AO63" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A64" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>60</v>
+        <v>98</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="K64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="L64" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="M64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M64" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O64" s="3" t="s">
-        <v>60</v>
+        <v>98</v>
+      </c>
+      <c r="O64" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="P64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="Q64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="R64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="S64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="T64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="U64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="V64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="W64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="X64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="Y64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
+      </c>
+      <c r="W64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="X64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y64" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z64" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA64" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB64" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="AC64" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AD64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE64" s="3" t="s">
-        <v>60</v>
+      <c r="AD64" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE64" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="AF64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="AG64" s="2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="AH64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="AI64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="AJ64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="AK64" s="3" t="s">
-        <v>60</v>
+        <v>98</v>
+      </c>
+      <c r="AK64" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="AL64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="AM64" s="2" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="AN64" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AO64" s="3" t="s">
-        <v>60</v>
+      <c r="AO64" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="65" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A65" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L65" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="T65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="U65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="W65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="X65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AI65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AK65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN65" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AO65" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A66" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D65" s="2" t="s">
+      <c r="B66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="N65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P65" s="2" t="s">
+      <c r="F66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="N66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="Q65" s="2" t="s">
+      <c r="Q66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="R65" s="2" t="s">
+      <c r="R66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="S65" s="2" t="s">
+      <c r="S66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="T65" s="2" t="s">
+      <c r="T66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="U65" s="2" t="s">
+      <c r="U66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="V65" s="2" t="s">
+      <c r="V66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="W65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="X65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z65" s="2" t="s">
+      <c r="W66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="X66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AA65" s="2" t="s">
+      <c r="AA66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AB65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AE65" s="2" t="s">
+      <c r="AB66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE66" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AF65" s="2" t="s">
+      <c r="AF66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AG65" s="2" t="s">
+      <c r="AG66" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AH65" s="2" t="s">
+      <c r="AH66" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="AI65" s="2" t="s">
+      <c r="AI66" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="AJ65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AK65" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AL65" s="2" t="s">
+      <c r="AJ66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AL66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AM65" s="2" t="s">
+      <c r="AM66" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AN65" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AO65" s="1" t="s">
+      <c r="AN66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AO66" s="1" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>